<commit_message>
trying from new mac
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F323C77C-2DEC-934E-8746-3BFF8BBEEA94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFF843A9-83FF-F148-984D-FA727A52D4D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5200" yWindow="500" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
+    <workbookView minimized="1" xWindow="5200" yWindow="500" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -108,7 +108,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -117,13 +117,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -140,10 +134,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,7 +549,7 @@
       <c r="A9" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
exp5 code change is test
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0B3D30-922E-F74F-AEA9-1638A6BCC4F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9858ECB5-CB12-D64C-A460-679F213F38C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
+    <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -592,14 +591,14 @@
       <c r="C2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>16</v>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>16</v>
+      <c r="F2" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>16</v>
@@ -621,8 +620,8 @@
       <c r="C3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>16</v>
+      <c r="D3" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>16</v>
@@ -650,8 +649,8 @@
       <c r="C4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>16</v>
+      <c r="D4" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>16</v>
@@ -679,7 +678,9 @@
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="5">
+        <v>10</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -696,7 +697,9 @@
       <c r="C6" s="5">
         <v>10</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="9">
+        <v>10</v>
+      </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -795,7 +798,7 @@
       <c r="B12" s="5">
         <v>10</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="5">
         <v>10</v>
       </c>
       <c r="D12" s="2"/>
@@ -812,8 +815,8 @@
       <c r="B13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>16</v>
+      <c r="C13" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
exp5 istest false and exp4 code fixed
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{918CE97A-14F3-6641-B518-953B6B241767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1582543A-6BC9-084E-8F07-1AFD1674AE6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
@@ -696,7 +696,7 @@
         <v>10</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="F5" s="10"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -806,7 +806,7 @@
       <c r="C11" s="5">
         <v>10</v>
       </c>
-      <c r="D11" s="10">
+      <c r="D11" s="9">
         <v>10</v>
       </c>
       <c r="E11" s="2"/>
@@ -825,7 +825,9 @@
       <c r="C12" s="5">
         <v>10</v>
       </c>
-      <c r="D12" s="2"/>
+      <c r="D12" s="9">
+        <v>10</v>
+      </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>

</xml_diff>

<commit_message>
exp4 exp5 list 2
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1582543A-6BC9-084E-8F07-1AFD1674AE6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E7DE04-2CC1-A64D-8259-D4E16BA801CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
@@ -608,8 +608,8 @@
       <c r="D2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>16</v>
+      <c r="E2" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>13</v>
@@ -637,11 +637,11 @@
       <c r="D3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>16</v>
+      <c r="E3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>16</v>
@@ -666,11 +666,11 @@
       <c r="D4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>16</v>
+      <c r="E4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>16</v>
@@ -695,8 +695,12 @@
       <c r="D5" s="5">
         <v>10</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="10"/>
+      <c r="E5" s="10">
+        <v>1</v>
+      </c>
+      <c r="F5" s="10">
+        <v>1</v>
+      </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -844,8 +848,8 @@
       <c r="C13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="8" t="s">
-        <v>16</v>
+      <c r="D13" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
exp4 exp5 list 3
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E7DE04-2CC1-A64D-8259-D4E16BA801CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71C5884-A02B-D346-B2A8-3E9CE56A38FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
@@ -695,11 +695,11 @@
       <c r="D5" s="5">
         <v>10</v>
       </c>
-      <c r="E5" s="10">
-        <v>1</v>
-      </c>
-      <c r="F5" s="10">
-        <v>1</v>
+      <c r="E5" s="5">
+        <v>10</v>
+      </c>
+      <c r="F5" s="5">
+        <v>10</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -718,8 +718,12 @@
       <c r="D6" s="5">
         <v>10</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="E6" s="5">
+        <v>10</v>
+      </c>
+      <c r="F6" s="5">
+        <v>10</v>
+      </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -737,8 +741,12 @@
       <c r="D7" s="5">
         <v>10</v>
       </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="E7" s="10">
+        <v>10</v>
+      </c>
+      <c r="F7" s="10">
+        <v>10</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>

</xml_diff>

<commit_message>
exp4 exp5 list 5
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71C5884-A02B-D346-B2A8-3E9CE56A38FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B6F1286-D5D1-214B-A524-5D337F026FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
@@ -741,10 +741,10 @@
       <c r="D7" s="5">
         <v>10</v>
       </c>
-      <c r="E7" s="10">
-        <v>10</v>
-      </c>
-      <c r="F7" s="10">
+      <c r="E7" s="5">
+        <v>10</v>
+      </c>
+      <c r="F7" s="5">
         <v>10</v>
       </c>
       <c r="G7" s="2"/>
@@ -764,8 +764,12 @@
       <c r="D8" s="5">
         <v>10</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="E8" s="10">
+        <v>10</v>
+      </c>
+      <c r="F8" s="10">
+        <v>10</v>
+      </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>

</xml_diff>

<commit_message>
exp4 exp5 list 6
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B6F1286-D5D1-214B-A524-5D337F026FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424E627E-7441-8C49-A314-F3A49047E63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
@@ -764,10 +764,10 @@
       <c r="D8" s="5">
         <v>10</v>
       </c>
-      <c r="E8" s="10">
-        <v>10</v>
-      </c>
-      <c r="F8" s="10">
+      <c r="E8" s="5">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5">
         <v>10</v>
       </c>
       <c r="G8" s="2"/>
@@ -787,8 +787,12 @@
       <c r="D9" s="9">
         <v>10</v>
       </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="E9" s="5">
+        <v>10</v>
+      </c>
+      <c r="F9" s="5">
+        <v>10</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -806,8 +810,12 @@
       <c r="D10" s="9">
         <v>10</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="E10" s="10">
+        <v>10</v>
+      </c>
+      <c r="F10" s="10">
+        <v>10</v>
+      </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>

</xml_diff>

<commit_message>
exp4 exp5 list 7
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424E627E-7441-8C49-A314-F3A49047E63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCEAAA36-8CBA-5C48-9BC5-BEC3F682CD9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
@@ -810,10 +810,10 @@
       <c r="D10" s="9">
         <v>10</v>
       </c>
-      <c r="E10" s="10">
-        <v>10</v>
-      </c>
-      <c r="F10" s="10">
+      <c r="E10" s="5">
+        <v>10</v>
+      </c>
+      <c r="F10" s="5">
         <v>10</v>
       </c>
       <c r="G10" s="2"/>
@@ -833,8 +833,12 @@
       <c r="D11" s="9">
         <v>10</v>
       </c>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="E11" s="10">
+        <v>10</v>
+      </c>
+      <c r="F11" s="10">
+        <v>10</v>
+      </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>

</xml_diff>

<commit_message>
changed code for q6,7,8
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCEAAA36-8CBA-5C48-9BC5-BEC3F682CD9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D4FF9B-F972-4843-9933-E6660C598488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
@@ -139,7 +139,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -167,12 +167,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA9D08E"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -228,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -239,7 +233,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -833,10 +826,10 @@
       <c r="D11" s="9">
         <v>10</v>
       </c>
-      <c r="E11" s="10">
-        <v>10</v>
-      </c>
-      <c r="F11" s="10">
+      <c r="E11" s="5">
+        <v>10</v>
+      </c>
+      <c r="F11" s="5">
         <v>10</v>
       </c>
       <c r="G11" s="2"/>
@@ -856,8 +849,12 @@
       <c r="D12" s="9">
         <v>10</v>
       </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="E12" s="5">
+        <v>10</v>
+      </c>
+      <c r="F12" s="5">
+        <v>10</v>
+      </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -875,11 +872,11 @@
       <c r="D13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>16</v>
+      <c r="E13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
istest false exp 6, 7, 8
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ishamody/Desktop/lbllm_behavioral/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D4FF9B-F972-4843-9933-E6660C598488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09FD0CBF-E679-9E48-8BEA-CF88649F5CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5200" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
+    <workbookView xWindow="5180" yWindow="680" windowWidth="21240" windowHeight="16020" xr2:uid="{5B3AD313-C567-A344-8F15-1E4D671AA27F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -222,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -230,7 +230,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -607,14 +606,14 @@
       <c r="F2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>16</v>
+      <c r="G2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -636,14 +635,14 @@
       <c r="F3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>16</v>
+      <c r="G3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -665,14 +664,14 @@
       <c r="F4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>16</v>
+      <c r="G4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -777,7 +776,7 @@
       <c r="C9" s="5">
         <v>10</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <v>10</v>
       </c>
       <c r="E9" s="5">
@@ -800,7 +799,7 @@
       <c r="C10" s="5">
         <v>10</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>10</v>
       </c>
       <c r="E10" s="5">
@@ -823,7 +822,7 @@
       <c r="C11" s="5">
         <v>10</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>10</v>
       </c>
       <c r="E11" s="5">
@@ -846,7 +845,7 @@
       <c r="C12" s="5">
         <v>10</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>10</v>
       </c>
       <c r="E12" s="5">
@@ -878,13 +877,13 @@
       <c r="F13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="I13" s="7" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>